<commit_message>
UI/UX enhancements: Fix admin sidebar bugs, normalize statistik header, improve peta UI, and optimize modal performance
</commit_message>
<xml_diff>
--- a/Data Penduduk Menurut Gender_101115.xlsx
+++ b/Data Penduduk Menurut Gender_101115.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\kangkung-peta\kangkung-peta\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0107319D-6A6A-4EFE-9B1B-5E74D73A0819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="75" windowWidth="15255" windowHeight="7935" firstSheet="1" activeTab="5"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Mutasi" sheetId="4" r:id="rId1"/>
@@ -14,7 +20,18 @@
     <sheet name="DATA KASUS" sheetId="15" r:id="rId5"/>
     <sheet name="DATA PENGELOLA" sheetId="16" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -348,8 +365,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -872,7 +889,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -882,8 +899,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -892,27 +907,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -941,67 +935,221 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1009,21 +1157,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1035,151 +1168,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1187,13 +1186,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1231,7 +1238,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1265,6 +1272,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1299,9 +1307,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1474,792 +1483,772 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:U22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.42578125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.44140625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" customWidth="1"/>
-    <col min="4" max="6" width="9.140625" style="1"/>
+    <col min="4" max="6" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" ht="17.25">
-      <c r="A2" s="67" t="s">
+    <row r="2" spans="1:21" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A2" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-      <c r="P2" s="67"/>
-      <c r="Q2" s="67"/>
-      <c r="R2" s="67"/>
-      <c r="S2" s="67"/>
-      <c r="T2" s="67"/>
-      <c r="U2" s="67"/>
-    </row>
-    <row r="3" spans="1:21" ht="17.25">
-      <c r="A3" s="67" t="s">
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="68"/>
+      <c r="P2" s="68"/>
+      <c r="Q2" s="68"/>
+      <c r="R2" s="68"/>
+      <c r="S2" s="68"/>
+      <c r="T2" s="68"/>
+      <c r="U2" s="68"/>
+    </row>
+    <row r="3" spans="1:21" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A3" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-    </row>
-    <row r="4" spans="1:21" ht="15.75" thickBot="1">
-      <c r="B4" s="16" t="s">
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
+      <c r="O3" s="68"/>
+      <c r="P3" s="68"/>
+      <c r="Q3" s="68"/>
+      <c r="R3" s="68"/>
+      <c r="S3" s="68"/>
+      <c r="T3" s="68"/>
+      <c r="U3" s="68"/>
+    </row>
+    <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-    </row>
-    <row r="5" spans="1:21" s="1" customFormat="1" ht="35.1" customHeight="1">
-      <c r="A5" s="68" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="69" t="s">
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+    </row>
+    <row r="5" spans="1:21" s="1" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="70" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="70" t="s">
+      <c r="C5" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="71" t="s">
+      <c r="D5" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="72"/>
-      <c r="F5" s="73"/>
-      <c r="G5" s="71" t="s">
+      <c r="E5" s="77"/>
+      <c r="F5" s="78"/>
+      <c r="G5" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="72"/>
-      <c r="I5" s="73"/>
-      <c r="J5" s="71" t="s">
+      <c r="H5" s="77"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="72"/>
-      <c r="L5" s="73"/>
-      <c r="M5" s="71" t="s">
+      <c r="K5" s="77"/>
+      <c r="L5" s="78"/>
+      <c r="M5" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="N5" s="72"/>
-      <c r="O5" s="73"/>
-      <c r="P5" s="74" t="s">
+      <c r="N5" s="77"/>
+      <c r="O5" s="78"/>
+      <c r="P5" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="Q5" s="75"/>
-      <c r="R5" s="76"/>
-      <c r="S5" s="74" t="s">
+      <c r="Q5" s="62"/>
+      <c r="R5" s="63"/>
+      <c r="S5" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="T5" s="75"/>
-      <c r="U5" s="76"/>
-    </row>
-    <row r="6" spans="1:21" s="1" customFormat="1" ht="21" customHeight="1">
-      <c r="A6" s="77"/>
-      <c r="B6" s="78"/>
-      <c r="C6" s="79"/>
-      <c r="D6" s="80" t="s">
+      <c r="T5" s="62"/>
+      <c r="U5" s="63"/>
+    </row>
+    <row r="6" spans="1:21" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="71"/>
+      <c r="B6" s="73"/>
+      <c r="C6" s="75"/>
+      <c r="D6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="81" t="s">
+      <c r="E6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="82" t="s">
+      <c r="F6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="80" t="s">
+      <c r="G6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="81" t="s">
+      <c r="H6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="82" t="s">
+      <c r="I6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="80" t="s">
+      <c r="J6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="81" t="s">
+      <c r="K6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="L6" s="82" t="s">
+      <c r="L6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="M6" s="80" t="s">
+      <c r="M6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="N6" s="81" t="s">
+      <c r="N6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="O6" s="82" t="s">
+      <c r="O6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="P6" s="80" t="s">
+      <c r="P6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="Q6" s="81" t="s">
+      <c r="Q6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="R6" s="82" t="s">
+      <c r="R6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="S6" s="80" t="s">
+      <c r="S6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="T6" s="81" t="s">
+      <c r="T6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="U6" s="82" t="s">
+      <c r="U6" s="36" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:21" s="3" customFormat="1" ht="9.75" customHeight="1">
-      <c r="A7" s="89">
+    <row r="7" spans="1:21" s="3" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="41">
         <v>1</v>
       </c>
-      <c r="B7" s="90">
+      <c r="B7" s="42">
         <v>2</v>
       </c>
-      <c r="C7" s="91">
+      <c r="C7" s="43">
         <v>3</v>
       </c>
-      <c r="D7" s="89">
+      <c r="D7" s="41">
         <v>4</v>
       </c>
-      <c r="E7" s="90">
+      <c r="E7" s="42">
         <v>5</v>
       </c>
-      <c r="F7" s="91">
+      <c r="F7" s="43">
         <v>6</v>
       </c>
-      <c r="G7" s="89">
+      <c r="G7" s="41">
         <v>7</v>
       </c>
-      <c r="H7" s="90">
+      <c r="H7" s="42">
         <v>8</v>
       </c>
-      <c r="I7" s="91">
+      <c r="I7" s="43">
         <v>9</v>
       </c>
-      <c r="J7" s="89">
+      <c r="J7" s="41">
         <v>10</v>
       </c>
-      <c r="K7" s="90">
+      <c r="K7" s="42">
         <v>11</v>
       </c>
-      <c r="L7" s="91">
+      <c r="L7" s="43">
         <v>12</v>
       </c>
-      <c r="M7" s="89">
+      <c r="M7" s="41">
         <v>13</v>
       </c>
-      <c r="N7" s="90">
+      <c r="N7" s="42">
         <v>14</v>
       </c>
-      <c r="O7" s="91">
+      <c r="O7" s="43">
         <v>15</v>
       </c>
-      <c r="P7" s="89">
+      <c r="P7" s="41">
         <v>16</v>
       </c>
-      <c r="Q7" s="90">
+      <c r="Q7" s="42">
         <v>17</v>
       </c>
-      <c r="R7" s="91">
+      <c r="R7" s="43">
         <v>18</v>
       </c>
-      <c r="S7" s="89">
+      <c r="S7" s="41">
         <v>19</v>
       </c>
-      <c r="T7" s="90">
+      <c r="T7" s="42">
         <v>20</v>
       </c>
-      <c r="U7" s="91">
+      <c r="U7" s="43">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="35.1" customHeight="1">
-      <c r="A8" s="80">
+    <row r="8" spans="1:21" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="34">
         <v>1</v>
       </c>
-      <c r="B8" s="83" t="s">
+      <c r="B8" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="82">
+      <c r="C8" s="36">
         <v>3643</v>
       </c>
-      <c r="D8" s="80">
+      <c r="D8" s="34">
         <v>5894</v>
       </c>
-      <c r="E8" s="81">
+      <c r="E8" s="35">
         <v>6925</v>
       </c>
-      <c r="F8" s="82">
+      <c r="F8" s="36">
         <f>SUM(D8:E8)</f>
         <v>12819</v>
       </c>
-      <c r="G8" s="80">
+      <c r="G8" s="34">
         <v>110</v>
       </c>
-      <c r="H8" s="81">
+      <c r="H8" s="35">
         <v>64</v>
       </c>
-      <c r="I8" s="82">
+      <c r="I8" s="36">
         <f>SUM(G8:H8)</f>
         <v>174</v>
       </c>
-      <c r="J8" s="80">
+      <c r="J8" s="34">
         <v>135</v>
       </c>
-      <c r="K8" s="81">
+      <c r="K8" s="35">
         <v>68</v>
       </c>
-      <c r="L8" s="82">
+      <c r="L8" s="36">
         <f>SUM(J8:K8)</f>
         <v>203</v>
       </c>
-      <c r="M8" s="80">
+      <c r="M8" s="34">
         <v>102</v>
       </c>
-      <c r="N8" s="81">
+      <c r="N8" s="35">
         <v>86</v>
       </c>
-      <c r="O8" s="82">
+      <c r="O8" s="36">
         <f>SUM(M8:N8)</f>
         <v>188</v>
       </c>
-      <c r="P8" s="80">
+      <c r="P8" s="34">
         <v>123</v>
       </c>
-      <c r="Q8" s="81">
+      <c r="Q8" s="35">
         <v>107</v>
       </c>
-      <c r="R8" s="82">
+      <c r="R8" s="36">
         <f>SUM(P8:Q8)</f>
         <v>230</v>
       </c>
-      <c r="S8" s="80">
+      <c r="S8" s="34">
         <f>D8+G8-J8+M8-P8</f>
         <v>5848</v>
       </c>
-      <c r="T8" s="81">
+      <c r="T8" s="35">
         <f>E8+H8-K8+N8-Q8</f>
         <v>6900</v>
       </c>
-      <c r="U8" s="82">
+      <c r="U8" s="36">
         <f>SUM(S8:T8)</f>
         <v>12748</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="35.1" customHeight="1">
-      <c r="A9" s="80">
+    <row r="9" spans="1:21" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="34">
         <v>2</v>
       </c>
-      <c r="B9" s="83" t="s">
+      <c r="B9" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="82">
+      <c r="C9" s="36">
         <v>4050</v>
       </c>
-      <c r="D9" s="80">
+      <c r="D9" s="34">
         <v>6966</v>
       </c>
-      <c r="E9" s="81">
+      <c r="E9" s="35">
         <v>6958</v>
       </c>
-      <c r="F9" s="82">
+      <c r="F9" s="36">
         <f t="shared" ref="F9:F10" si="0">SUM(D9:E9)</f>
         <v>13924</v>
       </c>
-      <c r="G9" s="80">
+      <c r="G9" s="34">
         <v>30</v>
       </c>
-      <c r="H9" s="81">
+      <c r="H9" s="35">
         <v>52</v>
       </c>
-      <c r="I9" s="82">
+      <c r="I9" s="36">
         <f t="shared" ref="I9:I12" si="1">SUM(G9:H9)</f>
         <v>82</v>
       </c>
-      <c r="J9" s="80">
+      <c r="J9" s="34">
         <v>58</v>
       </c>
-      <c r="K9" s="81">
+      <c r="K9" s="35">
         <v>44</v>
       </c>
-      <c r="L9" s="82">
+      <c r="L9" s="36">
         <f t="shared" ref="L9:L12" si="2">SUM(J9:K9)</f>
         <v>102</v>
       </c>
-      <c r="M9" s="80">
+      <c r="M9" s="34">
         <v>60</v>
       </c>
-      <c r="N9" s="81">
+      <c r="N9" s="35">
         <v>49</v>
       </c>
-      <c r="O9" s="82">
+      <c r="O9" s="36">
         <f t="shared" ref="O9:O12" si="3">SUM(M9:N9)</f>
         <v>109</v>
       </c>
-      <c r="P9" s="80">
+      <c r="P9" s="34">
         <v>56</v>
       </c>
-      <c r="Q9" s="81">
+      <c r="Q9" s="35">
         <v>62</v>
       </c>
-      <c r="R9" s="82">
+      <c r="R9" s="36">
         <f t="shared" ref="R9:R12" si="4">SUM(P9:Q9)</f>
         <v>118</v>
       </c>
-      <c r="S9" s="80">
+      <c r="S9" s="34">
         <f t="shared" ref="S9:T13" si="5">D9+G9-J9+M9-P9</f>
         <v>6942</v>
       </c>
-      <c r="T9" s="81">
+      <c r="T9" s="35">
         <f t="shared" si="5"/>
         <v>6953</v>
       </c>
-      <c r="U9" s="82">
+      <c r="U9" s="36">
         <f>SUM(S9:T9)</f>
         <v>13895</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="35.1" customHeight="1">
-      <c r="A10" s="80">
+    <row r="10" spans="1:21" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="34">
         <v>3</v>
       </c>
-      <c r="B10" s="83" t="s">
+      <c r="B10" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="82">
+      <c r="C10" s="36">
         <v>1423</v>
       </c>
-      <c r="D10" s="80">
+      <c r="D10" s="34">
         <v>2715</v>
       </c>
-      <c r="E10" s="81">
+      <c r="E10" s="35">
         <v>2474</v>
       </c>
-      <c r="F10" s="82">
+      <c r="F10" s="36">
         <f t="shared" si="0"/>
         <v>5189</v>
       </c>
-      <c r="G10" s="80">
+      <c r="G10" s="34">
         <v>6</v>
       </c>
-      <c r="H10" s="81">
+      <c r="H10" s="35">
         <v>4</v>
       </c>
-      <c r="I10" s="82">
+      <c r="I10" s="36">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="J10" s="80">
+      <c r="J10" s="34">
         <v>23</v>
       </c>
-      <c r="K10" s="81">
+      <c r="K10" s="35">
         <v>13</v>
       </c>
-      <c r="L10" s="82">
+      <c r="L10" s="36">
         <f t="shared" si="2"/>
         <v>36</v>
       </c>
-      <c r="M10" s="80">
-        <v>0</v>
-      </c>
-      <c r="N10" s="81">
-        <v>0</v>
-      </c>
-      <c r="O10" s="82">
+      <c r="M10" s="34">
+        <v>0</v>
+      </c>
+      <c r="N10" s="35">
+        <v>0</v>
+      </c>
+      <c r="O10" s="36">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P10" s="80">
+      <c r="P10" s="34">
         <v>30</v>
       </c>
-      <c r="Q10" s="81">
+      <c r="Q10" s="35">
         <v>21</v>
       </c>
-      <c r="R10" s="82">
+      <c r="R10" s="36">
         <f t="shared" si="4"/>
         <v>51</v>
       </c>
-      <c r="S10" s="80">
+      <c r="S10" s="34">
         <f t="shared" si="5"/>
         <v>2668</v>
       </c>
-      <c r="T10" s="81">
+      <c r="T10" s="35">
         <f t="shared" si="5"/>
         <v>2444</v>
       </c>
-      <c r="U10" s="82">
+      <c r="U10" s="36">
         <f>SUM(S10:T10)</f>
         <v>5112</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="35.1" customHeight="1">
-      <c r="A11" s="80">
+    <row r="11" spans="1:21" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="34">
         <v>4</v>
       </c>
-      <c r="B11" s="83" t="s">
+      <c r="B11" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="82">
+      <c r="C11" s="36">
         <v>2618</v>
       </c>
-      <c r="D11" s="80">
+      <c r="D11" s="34">
         <v>5276</v>
       </c>
-      <c r="E11" s="81">
+      <c r="E11" s="35">
         <v>5002</v>
       </c>
-      <c r="F11" s="82">
+      <c r="F11" s="36">
         <f>SUM(D11:E11)</f>
         <v>10278</v>
       </c>
-      <c r="G11" s="80">
+      <c r="G11" s="34">
         <v>19</v>
       </c>
-      <c r="H11" s="81">
+      <c r="H11" s="35">
         <v>21</v>
       </c>
-      <c r="I11" s="82">
+      <c r="I11" s="36">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="J11" s="80">
+      <c r="J11" s="34">
         <v>16</v>
       </c>
-      <c r="K11" s="81">
+      <c r="K11" s="35">
         <v>11</v>
       </c>
-      <c r="L11" s="82">
+      <c r="L11" s="36">
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
-      <c r="M11" s="80">
+      <c r="M11" s="34">
         <v>32</v>
       </c>
-      <c r="N11" s="81">
+      <c r="N11" s="35">
         <v>25</v>
       </c>
-      <c r="O11" s="82">
+      <c r="O11" s="36">
         <f t="shared" si="3"/>
         <v>57</v>
       </c>
-      <c r="P11" s="80">
+      <c r="P11" s="34">
         <v>14</v>
       </c>
-      <c r="Q11" s="81">
+      <c r="Q11" s="35">
         <v>8</v>
       </c>
-      <c r="R11" s="82">
+      <c r="R11" s="36">
         <f t="shared" si="4"/>
         <v>22</v>
       </c>
-      <c r="S11" s="80">
+      <c r="S11" s="34">
         <f t="shared" si="5"/>
         <v>5297</v>
       </c>
-      <c r="T11" s="81">
+      <c r="T11" s="35">
         <f t="shared" si="5"/>
         <v>5029</v>
       </c>
-      <c r="U11" s="82">
+      <c r="U11" s="36">
         <f>SUM(S11:T11)</f>
         <v>10326</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="35.1" customHeight="1">
-      <c r="A12" s="80">
+    <row r="12" spans="1:21" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="34">
         <v>5</v>
       </c>
-      <c r="B12" s="83" t="s">
+      <c r="B12" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="82">
+      <c r="C12" s="36">
         <v>2200</v>
       </c>
-      <c r="D12" s="80">
+      <c r="D12" s="34">
         <v>3788</v>
       </c>
-      <c r="E12" s="81">
+      <c r="E12" s="35">
         <v>3621</v>
       </c>
-      <c r="F12" s="82">
+      <c r="F12" s="36">
         <f t="shared" ref="F12" si="6">SUM(D12:E12)</f>
         <v>7409</v>
       </c>
-      <c r="G12" s="80">
-        <v>0</v>
-      </c>
-      <c r="H12" s="81">
+      <c r="G12" s="34">
+        <v>0</v>
+      </c>
+      <c r="H12" s="35">
         <v>3</v>
       </c>
-      <c r="I12" s="82">
+      <c r="I12" s="36">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J12" s="80">
+      <c r="J12" s="34">
         <v>34</v>
       </c>
-      <c r="K12" s="81">
+      <c r="K12" s="35">
         <v>26</v>
       </c>
-      <c r="L12" s="82">
+      <c r="L12" s="36">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
-      <c r="M12" s="80">
-        <v>0</v>
-      </c>
-      <c r="N12" s="81">
-        <v>0</v>
-      </c>
-      <c r="O12" s="82">
+      <c r="M12" s="34">
+        <v>0</v>
+      </c>
+      <c r="N12" s="35">
+        <v>0</v>
+      </c>
+      <c r="O12" s="36">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P12" s="80">
+      <c r="P12" s="34">
         <v>1</v>
       </c>
-      <c r="Q12" s="81">
+      <c r="Q12" s="35">
         <v>2</v>
       </c>
-      <c r="R12" s="82">
+      <c r="R12" s="36">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="S12" s="80">
+      <c r="S12" s="34">
         <f t="shared" si="5"/>
         <v>3753</v>
       </c>
-      <c r="T12" s="81">
+      <c r="T12" s="35">
         <f t="shared" si="5"/>
         <v>3596</v>
       </c>
-      <c r="U12" s="82">
+      <c r="U12" s="36">
         <f>SUM(S12:T12)</f>
         <v>7349</v>
       </c>
     </row>
-    <row r="13" spans="1:21" s="4" customFormat="1" ht="35.1" customHeight="1" thickBot="1">
-      <c r="A13" s="84" t="s">
+    <row r="13" spans="1:21" s="4" customFormat="1" ht="35.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="85"/>
-      <c r="C13" s="86">
+      <c r="B13" s="65"/>
+      <c r="C13" s="38">
         <f t="shared" ref="C13:N13" si="7">SUM(C8:C12)</f>
         <v>13934</v>
       </c>
-      <c r="D13" s="87">
+      <c r="D13" s="39">
         <f t="shared" si="7"/>
         <v>24639</v>
       </c>
-      <c r="E13" s="88">
+      <c r="E13" s="40">
         <f t="shared" si="7"/>
         <v>24980</v>
       </c>
-      <c r="F13" s="86">
+      <c r="F13" s="38">
         <f t="shared" si="7"/>
         <v>49619</v>
       </c>
-      <c r="G13" s="87">
+      <c r="G13" s="39">
         <f t="shared" si="7"/>
         <v>165</v>
       </c>
-      <c r="H13" s="88">
+      <c r="H13" s="40">
         <f t="shared" si="7"/>
         <v>144</v>
       </c>
-      <c r="I13" s="86">
+      <c r="I13" s="38">
         <f t="shared" si="7"/>
         <v>309</v>
       </c>
-      <c r="J13" s="87">
+      <c r="J13" s="39">
         <f t="shared" si="7"/>
         <v>266</v>
       </c>
-      <c r="K13" s="88">
+      <c r="K13" s="40">
         <f t="shared" si="7"/>
         <v>162</v>
       </c>
-      <c r="L13" s="86">
+      <c r="L13" s="38">
         <f t="shared" si="7"/>
         <v>428</v>
       </c>
-      <c r="M13" s="87">
+      <c r="M13" s="39">
         <f t="shared" si="7"/>
         <v>194</v>
       </c>
-      <c r="N13" s="88">
+      <c r="N13" s="40">
         <f t="shared" si="7"/>
         <v>160</v>
       </c>
-      <c r="O13" s="86">
+      <c r="O13" s="38">
         <f>SUM(M13:N13)</f>
         <v>354</v>
       </c>
-      <c r="P13" s="87">
+      <c r="P13" s="39">
         <f>SUM(P8:P12)</f>
         <v>224</v>
       </c>
-      <c r="Q13" s="88">
+      <c r="Q13" s="40">
         <f>SUM(Q8:Q12)</f>
         <v>200</v>
       </c>
-      <c r="R13" s="86">
+      <c r="R13" s="38">
         <f>SUM(R8:R12)</f>
         <v>424</v>
       </c>
-      <c r="S13" s="87">
+      <c r="S13" s="39">
         <f t="shared" si="5"/>
         <v>24508</v>
       </c>
-      <c r="T13" s="88">
+      <c r="T13" s="40">
         <f t="shared" si="5"/>
         <v>24922</v>
       </c>
-      <c r="U13" s="86">
+      <c r="U13" s="38">
         <f>SUM(U8:U12)</f>
         <v>49430</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
-      <c r="I14" s="5"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="5"/>
-      <c r="U14" s="5"/>
-    </row>
-    <row r="15" spans="1:21" ht="15.75">
-      <c r="O15" s="111" t="s">
+    <row r="15" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O15" s="66" t="s">
         <v>100</v>
       </c>
-      <c r="P15" s="111"/>
-      <c r="Q15" s="111"/>
-      <c r="R15" s="111"/>
-      <c r="S15" s="111"/>
-      <c r="T15" s="111"/>
-      <c r="U15" s="111"/>
-    </row>
-    <row r="16" spans="1:21" ht="15.75">
-      <c r="O16" s="111" t="s">
+      <c r="P15" s="66"/>
+      <c r="Q15" s="66"/>
+      <c r="R15" s="66"/>
+      <c r="S15" s="66"/>
+      <c r="T15" s="66"/>
+      <c r="U15" s="66"/>
+    </row>
+    <row r="16" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O16" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="P16" s="111"/>
-      <c r="Q16" s="111"/>
-      <c r="R16" s="111"/>
-      <c r="S16" s="111"/>
-      <c r="T16" s="111"/>
-      <c r="U16" s="111"/>
-    </row>
-    <row r="17" spans="15:21" ht="15.75">
-      <c r="O17" s="112"/>
-      <c r="P17" s="112"/>
-      <c r="Q17" s="112"/>
-      <c r="R17" s="112"/>
-      <c r="S17" s="112"/>
-      <c r="T17" s="112"/>
-      <c r="U17" s="112"/>
-    </row>
-    <row r="18" spans="15:21" ht="15.75">
-      <c r="O18" s="112"/>
-      <c r="P18" s="112"/>
-      <c r="Q18" s="112"/>
-      <c r="R18" s="112"/>
-      <c r="S18" s="112"/>
-      <c r="T18" s="112"/>
-      <c r="U18" s="112"/>
-    </row>
-    <row r="19" spans="15:21" ht="15.75">
-      <c r="O19" s="112"/>
-      <c r="P19" s="112"/>
-      <c r="Q19" s="112"/>
-      <c r="R19" s="112"/>
-      <c r="S19" s="112"/>
-      <c r="T19" s="112"/>
-      <c r="U19" s="112"/>
-    </row>
-    <row r="20" spans="15:21" ht="15.75">
-      <c r="O20" s="112"/>
-      <c r="P20" s="112"/>
-      <c r="Q20" s="112"/>
-      <c r="R20" s="112"/>
-      <c r="S20" s="112"/>
-      <c r="T20" s="112"/>
-      <c r="U20" s="112"/>
-    </row>
-    <row r="21" spans="15:21" ht="15.75">
-      <c r="O21" s="113" t="s">
+      <c r="P16" s="66"/>
+      <c r="Q16" s="66"/>
+      <c r="R16" s="66"/>
+      <c r="S16" s="66"/>
+      <c r="T16" s="66"/>
+      <c r="U16" s="66"/>
+    </row>
+    <row r="17" spans="15:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O17" s="56"/>
+      <c r="P17" s="56"/>
+      <c r="Q17" s="56"/>
+      <c r="R17" s="56"/>
+      <c r="S17" s="56"/>
+      <c r="T17" s="56"/>
+      <c r="U17" s="56"/>
+    </row>
+    <row r="18" spans="15:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O18" s="56"/>
+      <c r="P18" s="56"/>
+      <c r="Q18" s="56"/>
+      <c r="R18" s="56"/>
+      <c r="S18" s="56"/>
+      <c r="T18" s="56"/>
+      <c r="U18" s="56"/>
+    </row>
+    <row r="19" spans="15:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O19" s="56"/>
+      <c r="P19" s="56"/>
+      <c r="Q19" s="56"/>
+      <c r="R19" s="56"/>
+      <c r="S19" s="56"/>
+      <c r="T19" s="56"/>
+      <c r="U19" s="56"/>
+    </row>
+    <row r="20" spans="15:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O20" s="56"/>
+      <c r="P20" s="56"/>
+      <c r="Q20" s="56"/>
+      <c r="R20" s="56"/>
+      <c r="S20" s="56"/>
+      <c r="T20" s="56"/>
+      <c r="U20" s="56"/>
+    </row>
+    <row r="21" spans="15:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O21" s="67" t="s">
         <v>97</v>
       </c>
-      <c r="P21" s="113"/>
-      <c r="Q21" s="113"/>
-      <c r="R21" s="113"/>
-      <c r="S21" s="113"/>
-      <c r="T21" s="113"/>
-      <c r="U21" s="113"/>
-    </row>
-    <row r="22" spans="15:21" ht="15.75">
-      <c r="O22" s="111" t="s">
+      <c r="P21" s="67"/>
+      <c r="Q21" s="67"/>
+      <c r="R21" s="67"/>
+      <c r="S21" s="67"/>
+      <c r="T21" s="67"/>
+      <c r="U21" s="67"/>
+    </row>
+    <row r="22" spans="15:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O22" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="P22" s="111"/>
-      <c r="Q22" s="111"/>
-      <c r="R22" s="111"/>
-      <c r="S22" s="111"/>
-      <c r="T22" s="111"/>
-      <c r="U22" s="111"/>
+      <c r="P22" s="66"/>
+      <c r="Q22" s="66"/>
+      <c r="R22" s="66"/>
+      <c r="S22" s="66"/>
+      <c r="T22" s="66"/>
+      <c r="U22" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="P5:R5"/>
-    <mergeCell ref="S5:U5"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="O15:U15"/>
-    <mergeCell ref="O16:U16"/>
     <mergeCell ref="O21:U21"/>
     <mergeCell ref="O22:U22"/>
     <mergeCell ref="A2:U2"/>
@@ -2272,84 +2261,88 @@
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="J5:L5"/>
     <mergeCell ref="M5:O5"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="S5:U5"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="O15:U15"/>
+    <mergeCell ref="O16:U16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="65" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="65" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:S36"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A2:S29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" customWidth="1"/>
+    <col min="7" max="7" width="9.44140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:19">
-      <c r="A2" s="30" t="s">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A2" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-    </row>
-    <row r="3" spans="1:19">
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:19">
-      <c r="A4" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="35" t="s">
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A4" s="84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="81" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="87" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="35" t="s">
+      <c r="D4" s="88"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="81" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="19"/>
-    </row>
-    <row r="5" spans="1:19">
-      <c r="A5" s="32"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="20" t="s">
+      <c r="H4" s="10"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A5" s="85"/>
+      <c r="B5" s="82"/>
+      <c r="C5" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="36"/>
-      <c r="H5" s="20" t="s">
+      <c r="G5" s="82"/>
+      <c r="H5" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" t="s">
         <v>53</v>
       </c>
-      <c r="K5" s="6"/>
       <c r="L5" t="s">
         <v>54</v>
       </c>
@@ -2363,19 +2356,19 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:19">
-      <c r="A6" s="33"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="22" t="s">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A6" s="86"/>
+      <c r="B6" s="83"/>
+      <c r="C6" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22" t="s">
+      <c r="D6" s="13"/>
+      <c r="E6" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="21"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="21"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="12"/>
       <c r="J6" t="s">
         <v>5</v>
       </c>
@@ -2407,28 +2400,28 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
-      <c r="A7" s="104">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A7" s="49">
         <v>1</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="43">
+      <c r="C7" s="22">
         <f>J7+L7+N7+P7+R7</f>
         <v>1575</v>
       </c>
-      <c r="D7" s="105"/>
-      <c r="E7" s="43">
+      <c r="D7" s="50"/>
+      <c r="E7" s="22">
         <f>K7+M7+O7+Q7+S7</f>
         <v>1397</v>
       </c>
-      <c r="F7" s="106"/>
-      <c r="G7" s="45">
+      <c r="F7" s="51"/>
+      <c r="G7" s="7">
         <f>C7+E7</f>
         <v>2972</v>
       </c>
-      <c r="H7" s="106"/>
+      <c r="H7" s="51"/>
       <c r="J7">
         <v>480</v>
       </c>
@@ -2460,28 +2453,28 @@
         <v>244</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
-      <c r="A8" s="43">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A8" s="22">
         <v>2</v>
       </c>
-      <c r="B8" s="107" t="s">
+      <c r="B8" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="43">
+      <c r="C8" s="22">
         <f t="shared" ref="C8:C19" si="0">J8+L8+N8+P8+R8</f>
         <v>1750</v>
       </c>
-      <c r="D8" s="105"/>
-      <c r="E8" s="43">
+      <c r="D8" s="50"/>
+      <c r="E8" s="22">
         <f t="shared" ref="E8:E19" si="1">K8+M8+O8+Q8+S8</f>
         <v>1667</v>
       </c>
-      <c r="F8" s="106"/>
-      <c r="G8" s="45">
+      <c r="F8" s="51"/>
+      <c r="G8" s="7">
         <f t="shared" ref="G8:G19" si="2">C8+E8</f>
         <v>3417</v>
       </c>
-      <c r="H8" s="106"/>
+      <c r="H8" s="51"/>
       <c r="J8">
         <v>535</v>
       </c>
@@ -2513,28 +2506,28 @@
         <v>187</v>
       </c>
     </row>
-    <row r="9" spans="1:19">
-      <c r="A9" s="43">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A9" s="22">
         <v>3</v>
       </c>
-      <c r="B9" s="108" t="s">
+      <c r="B9" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="43">
+      <c r="C9" s="22">
         <f t="shared" si="0"/>
         <v>1963</v>
       </c>
-      <c r="D9" s="105"/>
-      <c r="E9" s="43">
+      <c r="D9" s="50"/>
+      <c r="E9" s="22">
         <f t="shared" si="1"/>
         <v>1885</v>
       </c>
-      <c r="F9" s="106"/>
-      <c r="G9" s="45">
+      <c r="F9" s="51"/>
+      <c r="G9" s="7">
         <f t="shared" si="2"/>
         <v>3848</v>
       </c>
-      <c r="H9" s="106"/>
+      <c r="H9" s="51"/>
       <c r="J9">
         <v>466</v>
       </c>
@@ -2566,28 +2559,28 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
-      <c r="A10" s="43">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A10" s="22">
         <v>4</v>
       </c>
-      <c r="B10" s="109" t="s">
+      <c r="B10" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="43">
+      <c r="C10" s="22">
         <f t="shared" si="0"/>
         <v>2039</v>
       </c>
-      <c r="D10" s="105"/>
-      <c r="E10" s="43">
+      <c r="D10" s="50"/>
+      <c r="E10" s="22">
         <f t="shared" si="1"/>
         <v>1736</v>
       </c>
-      <c r="F10" s="106"/>
-      <c r="G10" s="45">
+      <c r="F10" s="51"/>
+      <c r="G10" s="7">
         <f t="shared" si="2"/>
         <v>3775</v>
       </c>
-      <c r="H10" s="106"/>
+      <c r="H10" s="51"/>
       <c r="J10">
         <v>584</v>
       </c>
@@ -2619,28 +2612,28 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:19">
-      <c r="A11" s="43">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A11" s="22">
         <v>5</v>
       </c>
-      <c r="B11" s="109" t="s">
+      <c r="B11" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="43">
+      <c r="C11" s="22">
         <f t="shared" si="0"/>
         <v>2161</v>
       </c>
-      <c r="D11" s="105"/>
-      <c r="E11" s="43">
+      <c r="D11" s="50"/>
+      <c r="E11" s="22">
         <f t="shared" si="1"/>
         <v>2012</v>
       </c>
-      <c r="F11" s="106"/>
-      <c r="G11" s="45">
+      <c r="F11" s="51"/>
+      <c r="G11" s="7">
         <f t="shared" si="2"/>
         <v>4173</v>
       </c>
-      <c r="H11" s="106"/>
+      <c r="H11" s="51"/>
       <c r="J11">
         <v>439</v>
       </c>
@@ -2672,28 +2665,28 @@
         <v>447</v>
       </c>
     </row>
-    <row r="12" spans="1:19">
-      <c r="A12" s="43">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A12" s="22">
         <v>6</v>
       </c>
-      <c r="B12" s="109" t="s">
+      <c r="B12" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="43">
+      <c r="C12" s="22">
         <f t="shared" si="0"/>
         <v>2058</v>
       </c>
-      <c r="D12" s="105"/>
-      <c r="E12" s="43">
+      <c r="D12" s="50"/>
+      <c r="E12" s="22">
         <f t="shared" si="1"/>
         <v>1984</v>
       </c>
-      <c r="F12" s="106"/>
-      <c r="G12" s="45">
+      <c r="F12" s="51"/>
+      <c r="G12" s="7">
         <f t="shared" si="2"/>
         <v>4042</v>
       </c>
-      <c r="H12" s="106"/>
+      <c r="H12" s="51"/>
       <c r="J12">
         <v>582</v>
       </c>
@@ -2725,28 +2718,28 @@
         <v>324</v>
       </c>
     </row>
-    <row r="13" spans="1:19">
-      <c r="A13" s="43">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A13" s="22">
         <v>7</v>
       </c>
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="43">
+      <c r="C13" s="22">
         <f t="shared" si="0"/>
         <v>2066</v>
       </c>
-      <c r="D13" s="105"/>
-      <c r="E13" s="43">
+      <c r="D13" s="50"/>
+      <c r="E13" s="22">
         <f t="shared" si="1"/>
         <v>1965</v>
       </c>
-      <c r="F13" s="106"/>
-      <c r="G13" s="45">
+      <c r="F13" s="51"/>
+      <c r="G13" s="7">
         <f t="shared" si="2"/>
         <v>4031</v>
       </c>
-      <c r="H13" s="106"/>
+      <c r="H13" s="51"/>
       <c r="J13">
         <v>572</v>
       </c>
@@ -2778,28 +2771,28 @@
         <v>422</v>
       </c>
     </row>
-    <row r="14" spans="1:19">
-      <c r="A14" s="43">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A14" s="22">
         <v>8</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="22">
         <f t="shared" si="0"/>
         <v>1963</v>
       </c>
-      <c r="D14" s="105"/>
-      <c r="E14" s="43">
+      <c r="D14" s="50"/>
+      <c r="E14" s="22">
         <f t="shared" si="1"/>
         <v>2106</v>
       </c>
-      <c r="F14" s="106"/>
-      <c r="G14" s="45">
+      <c r="F14" s="51"/>
+      <c r="G14" s="7">
         <f t="shared" si="2"/>
         <v>4069</v>
       </c>
-      <c r="H14" s="106"/>
+      <c r="H14" s="51"/>
       <c r="J14">
         <v>473</v>
       </c>
@@ -2831,28 +2824,28 @@
         <v>288</v>
       </c>
     </row>
-    <row r="15" spans="1:19">
-      <c r="A15" s="43">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A15" s="22">
         <v>9</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="22">
         <f t="shared" si="0"/>
         <v>2167</v>
       </c>
-      <c r="D15" s="105"/>
-      <c r="E15" s="43">
+      <c r="D15" s="50"/>
+      <c r="E15" s="22">
         <f t="shared" si="1"/>
         <v>2123</v>
       </c>
-      <c r="F15" s="106"/>
-      <c r="G15" s="45">
+      <c r="F15" s="51"/>
+      <c r="G15" s="7">
         <f t="shared" si="2"/>
         <v>4290</v>
       </c>
-      <c r="H15" s="106"/>
+      <c r="H15" s="51"/>
       <c r="J15">
         <v>438</v>
       </c>
@@ -2884,28 +2877,28 @@
         <v>322</v>
       </c>
     </row>
-    <row r="16" spans="1:19">
-      <c r="A16" s="43">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A16" s="22">
         <v>10</v>
       </c>
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="43">
+      <c r="C16" s="22">
         <f t="shared" si="0"/>
         <v>2177</v>
       </c>
-      <c r="D16" s="105"/>
-      <c r="E16" s="43">
+      <c r="D16" s="50"/>
+      <c r="E16" s="22">
         <f t="shared" si="1"/>
         <v>1978</v>
       </c>
-      <c r="F16" s="106"/>
-      <c r="G16" s="45">
+      <c r="F16" s="51"/>
+      <c r="G16" s="7">
         <f t="shared" si="2"/>
         <v>4155</v>
       </c>
-      <c r="H16" s="106"/>
+      <c r="H16" s="51"/>
       <c r="J16">
         <v>439</v>
       </c>
@@ -2937,28 +2930,28 @@
         <v>425</v>
       </c>
     </row>
-    <row r="17" spans="1:19">
-      <c r="A17" s="43">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A17" s="22">
         <v>11</v>
       </c>
-      <c r="B17" s="43" t="s">
+      <c r="B17" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="43">
+      <c r="C17" s="22">
         <f t="shared" si="0"/>
         <v>2031</v>
       </c>
-      <c r="D17" s="105"/>
-      <c r="E17" s="43">
+      <c r="D17" s="50"/>
+      <c r="E17" s="22">
         <f t="shared" si="1"/>
         <v>1708</v>
       </c>
-      <c r="F17" s="106"/>
-      <c r="G17" s="45">
+      <c r="F17" s="51"/>
+      <c r="G17" s="7">
         <f t="shared" si="2"/>
         <v>3739</v>
       </c>
-      <c r="H17" s="106"/>
+      <c r="H17" s="51"/>
       <c r="J17">
         <v>594</v>
       </c>
@@ -2990,29 +2983,29 @@
         <v>345</v>
       </c>
     </row>
-    <row r="18" spans="1:19">
-      <c r="A18" s="43">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A18" s="22">
         <v>12</v>
       </c>
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="43">
+      <c r="C18" s="22">
         <f t="shared" si="0"/>
         <v>1816</v>
       </c>
-      <c r="D18" s="105"/>
-      <c r="E18" s="43">
+      <c r="D18" s="50"/>
+      <c r="E18" s="22">
         <f t="shared" si="1"/>
         <v>1754</v>
       </c>
-      <c r="F18" s="106"/>
-      <c r="G18" s="45">
+      <c r="F18" s="51"/>
+      <c r="G18" s="7">
         <f t="shared" si="2"/>
         <v>3570</v>
       </c>
-      <c r="H18" s="106"/>
-      <c r="I18" s="25"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="16"/>
       <c r="J18">
         <v>459</v>
       </c>
@@ -3044,29 +3037,29 @@
         <v>421</v>
       </c>
     </row>
-    <row r="19" spans="1:19">
-      <c r="A19" s="43">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" s="22">
         <v>13</v>
       </c>
-      <c r="B19" s="43" t="s">
+      <c r="B19" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="43">
+      <c r="C19" s="22">
         <f t="shared" si="0"/>
         <v>1781</v>
       </c>
-      <c r="D19" s="105"/>
-      <c r="E19" s="43">
+      <c r="D19" s="50"/>
+      <c r="E19" s="22">
         <f t="shared" si="1"/>
         <v>1859</v>
       </c>
-      <c r="F19" s="106"/>
-      <c r="G19" s="45">
+      <c r="F19" s="51"/>
+      <c r="G19" s="7">
         <f t="shared" si="2"/>
         <v>3640</v>
       </c>
-      <c r="H19" s="110"/>
-      <c r="I19" s="25"/>
+      <c r="H19" s="55"/>
+      <c r="I19" s="16"/>
       <c r="J19">
         <v>484</v>
       </c>
@@ -3098,86 +3091,62 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:19">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="27">
+      <c r="C20" s="18">
         <f>SUM(C7:C19)</f>
         <v>25547</v>
       </c>
-      <c r="D20" s="23"/>
-      <c r="E20" s="28">
+      <c r="D20" s="14"/>
+      <c r="E20" s="19">
         <f>SUM(E7:E19)</f>
         <v>24174</v>
       </c>
-      <c r="F20" s="24"/>
-      <c r="G20" s="103">
+      <c r="F20" s="15"/>
+      <c r="G20" s="48">
         <f>SUM(G7:G19)</f>
         <v>49721</v>
       </c>
-      <c r="H20" s="29"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="6"/>
-    </row>
-    <row r="21" spans="1:19">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-    </row>
-    <row r="22" spans="1:19">
-      <c r="D22" s="11" t="s">
+      <c r="H20" s="20"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="D22" s="79" t="s">
         <v>104</v>
       </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-    </row>
-    <row r="23" spans="1:19">
-      <c r="D23" s="11" t="s">
+      <c r="E22" s="79"/>
+      <c r="F22" s="79"/>
+      <c r="G22" s="79"/>
+      <c r="H22" s="79"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="D23" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-    </row>
-    <row r="28" spans="1:19">
-      <c r="D28" s="10" t="s">
+      <c r="E23" s="79"/>
+      <c r="F23" s="79"/>
+      <c r="G23" s="79"/>
+      <c r="H23" s="79"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="D28" s="80" t="s">
         <v>106</v>
       </c>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-    </row>
-    <row r="29" spans="1:19">
-      <c r="D29" s="11" t="s">
+      <c r="E28" s="80"/>
+      <c r="F28" s="80"/>
+      <c r="G28" s="80"/>
+      <c r="H28" s="80"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="D29" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-    </row>
-    <row r="35" spans="9:11">
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-    </row>
-    <row r="36" spans="9:11">
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
+      <c r="E29" s="79"/>
+      <c r="F29" s="79"/>
+      <c r="G29" s="79"/>
+      <c r="H29" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3192,788 +3161,789 @@
     <mergeCell ref="G4:G6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:O29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" customWidth="1"/>
-    <col min="3" max="4" width="13.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" customWidth="1"/>
+    <col min="3" max="4" width="13.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="14" style="1" customWidth="1"/>
-    <col min="6" max="15" width="9.140625" style="1"/>
+    <col min="6" max="15" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:15">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="80" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-    </row>
-    <row r="5" spans="1:15" ht="15.75" thickBot="1">
-      <c r="A5" s="40"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" thickTop="1">
-      <c r="A6" s="59" t="s">
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+    </row>
+    <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="99" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="60"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="47" t="s">
+      <c r="B6" s="100"/>
+      <c r="C6" s="100"/>
+      <c r="D6" s="100"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="90" t="s">
         <v>59</v>
       </c>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="48"/>
-      <c r="N6" s="48"/>
-      <c r="O6" s="49"/>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="A7" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="15" t="s">
+      <c r="G6" s="91"/>
+      <c r="H6" s="91"/>
+      <c r="I6" s="91"/>
+      <c r="J6" s="91"/>
+      <c r="K6" s="91"/>
+      <c r="L6" s="91"/>
+      <c r="M6" s="91"/>
+      <c r="N6" s="91"/>
+      <c r="O6" s="92"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="60" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="E7" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="50" t="s">
+      <c r="F7" s="93" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="46" t="s">
+      <c r="G7" s="94"/>
+      <c r="H7" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="14"/>
-      <c r="J7" s="46" t="s">
+      <c r="I7" s="94"/>
+      <c r="J7" s="95" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="14"/>
-      <c r="L7" s="46" t="s">
+      <c r="K7" s="94"/>
+      <c r="L7" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="M7" s="14"/>
-      <c r="N7" s="46" t="s">
+      <c r="M7" s="94"/>
+      <c r="N7" s="95" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="51"/>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="A8" s="62"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="63"/>
-      <c r="F8" s="52" t="s">
+      <c r="O7" s="96"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="97"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="98"/>
+      <c r="F8" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L8" s="8" t="s">
+      <c r="L8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="M8" s="8" t="s">
+      <c r="M8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="N8" s="8" t="s">
+      <c r="N8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="O8" s="53" t="s">
+      <c r="O8" s="25" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
-      <c r="A9" s="64">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="31">
         <v>1</v>
       </c>
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="45">
+      <c r="C9" s="7">
         <f>F9+H9+J9+L9+N9</f>
         <v>154</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="7">
         <f>G9+I9+K9+M9+O9</f>
         <v>109</v>
       </c>
-      <c r="E9" s="55">
+      <c r="E9" s="27">
         <f>C9+D9</f>
         <v>263</v>
       </c>
-      <c r="F9" s="54">
+      <c r="F9" s="26">
         <v>11</v>
       </c>
-      <c r="G9" s="45">
+      <c r="G9" s="7">
         <v>17</v>
       </c>
-      <c r="H9" s="45">
+      <c r="H9" s="7">
         <v>41</v>
       </c>
-      <c r="I9" s="45">
+      <c r="I9" s="7">
         <v>31</v>
       </c>
-      <c r="J9" s="45">
+      <c r="J9" s="7">
         <v>27</v>
       </c>
-      <c r="K9" s="45">
+      <c r="K9" s="7">
         <v>10</v>
       </c>
-      <c r="L9" s="45">
+      <c r="L9" s="7">
         <v>54</v>
       </c>
-      <c r="M9" s="45">
+      <c r="M9" s="7">
         <v>28</v>
       </c>
-      <c r="N9" s="45">
+      <c r="N9" s="7">
         <v>21</v>
       </c>
-      <c r="O9" s="55">
+      <c r="O9" s="27">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
-      <c r="A10" s="64">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="31">
         <v>2</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="45">
+      <c r="C10" s="7">
         <f t="shared" ref="C10:C19" si="0">F10+H10+J10+L10+N10</f>
         <v>10273</v>
       </c>
-      <c r="D10" s="45">
+      <c r="D10" s="7">
         <f t="shared" ref="D10:D19" si="1">G10+I10+K10+M10+O10</f>
         <v>3054</v>
       </c>
-      <c r="E10" s="55">
+      <c r="E10" s="27">
         <f t="shared" ref="E10:E19" si="2">C10+D10</f>
         <v>13327</v>
       </c>
-      <c r="F10" s="54">
+      <c r="F10" s="26">
         <v>1995</v>
       </c>
-      <c r="G10" s="45">
+      <c r="G10" s="7">
         <v>459</v>
       </c>
-      <c r="H10" s="45">
+      <c r="H10" s="7">
         <v>3707</v>
       </c>
-      <c r="I10" s="45">
+      <c r="I10" s="7">
         <v>564</v>
       </c>
-      <c r="J10" s="45">
+      <c r="J10" s="7">
         <v>518</v>
       </c>
-      <c r="K10" s="45">
+      <c r="K10" s="7">
         <v>46</v>
       </c>
-      <c r="L10" s="45">
+      <c r="L10" s="7">
         <v>2577</v>
       </c>
-      <c r="M10" s="45">
+      <c r="M10" s="7">
         <v>1570</v>
       </c>
-      <c r="N10" s="45">
+      <c r="N10" s="7">
         <v>1476</v>
       </c>
-      <c r="O10" s="55">
+      <c r="O10" s="27">
         <v>415</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
-      <c r="A11" s="64">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="31">
         <v>3</v>
       </c>
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="45">
+      <c r="C11" s="7">
         <f t="shared" si="0"/>
         <v>1430</v>
       </c>
-      <c r="D11" s="45">
+      <c r="D11" s="7">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="E11" s="55">
+      <c r="E11" s="27">
         <f t="shared" si="2"/>
         <v>1490</v>
       </c>
-      <c r="F11" s="54">
+      <c r="F11" s="26">
         <v>1245</v>
       </c>
-      <c r="G11" s="45">
-        <v>0</v>
-      </c>
-      <c r="H11" s="45">
+      <c r="G11" s="7">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7">
         <v>31</v>
       </c>
-      <c r="I11" s="45">
-        <v>0</v>
-      </c>
-      <c r="J11" s="45">
+      <c r="I11" s="7">
+        <v>0</v>
+      </c>
+      <c r="J11" s="7">
         <v>1</v>
       </c>
-      <c r="K11" s="45">
-        <v>0</v>
-      </c>
-      <c r="L11" s="45">
+      <c r="K11" s="7">
+        <v>0</v>
+      </c>
+      <c r="L11" s="7">
         <v>153</v>
       </c>
-      <c r="M11" s="45">
+      <c r="M11" s="7">
         <v>60</v>
       </c>
-      <c r="N11" s="45">
-        <v>0</v>
-      </c>
-      <c r="O11" s="55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
-      <c r="A12" s="64">
+      <c r="N11" s="7">
+        <v>0</v>
+      </c>
+      <c r="O11" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="31">
         <v>4</v>
       </c>
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="45">
+      <c r="C12" s="7">
         <f t="shared" si="0"/>
         <v>1188</v>
       </c>
-      <c r="D12" s="45">
+      <c r="D12" s="7">
         <f t="shared" si="1"/>
         <v>424</v>
       </c>
-      <c r="E12" s="55">
+      <c r="E12" s="27">
         <f t="shared" si="2"/>
         <v>1612</v>
       </c>
-      <c r="F12" s="54">
+      <c r="F12" s="26">
         <v>409</v>
       </c>
-      <c r="G12" s="45">
+      <c r="G12" s="7">
         <v>189</v>
       </c>
-      <c r="H12" s="45">
+      <c r="H12" s="7">
         <v>278</v>
       </c>
-      <c r="I12" s="45">
+      <c r="I12" s="7">
         <v>54</v>
       </c>
-      <c r="J12" s="45">
+      <c r="J12" s="7">
         <v>174</v>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="7">
         <v>57</v>
       </c>
-      <c r="L12" s="45">
+      <c r="L12" s="7">
         <v>327</v>
       </c>
-      <c r="M12" s="45">
+      <c r="M12" s="7">
         <v>124</v>
       </c>
-      <c r="N12" s="45">
-        <v>0</v>
-      </c>
-      <c r="O12" s="55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" s="64">
+      <c r="N12" s="7">
+        <v>0</v>
+      </c>
+      <c r="O12" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="31">
         <v>5</v>
       </c>
-      <c r="B13" s="44" t="s">
+      <c r="B13" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="45">
+      <c r="C13" s="7">
         <f t="shared" si="0"/>
         <v>1797</v>
       </c>
-      <c r="D13" s="45">
+      <c r="D13" s="7">
         <f t="shared" si="1"/>
         <v>1269</v>
       </c>
-      <c r="E13" s="55">
+      <c r="E13" s="27">
         <f t="shared" si="2"/>
         <v>3066</v>
       </c>
-      <c r="F13" s="54">
+      <c r="F13" s="26">
         <v>572</v>
       </c>
-      <c r="G13" s="45">
+      <c r="G13" s="7">
         <v>242</v>
       </c>
-      <c r="H13" s="45">
+      <c r="H13" s="7">
         <v>299</v>
       </c>
-      <c r="I13" s="45">
+      <c r="I13" s="7">
         <v>274</v>
       </c>
-      <c r="J13" s="45">
+      <c r="J13" s="7">
         <v>76</v>
       </c>
-      <c r="K13" s="45">
+      <c r="K13" s="7">
         <v>59</v>
       </c>
-      <c r="L13" s="45">
+      <c r="L13" s="7">
         <v>813</v>
       </c>
-      <c r="M13" s="45">
+      <c r="M13" s="7">
         <v>525</v>
       </c>
-      <c r="N13" s="45">
+      <c r="N13" s="7">
         <v>37</v>
       </c>
-      <c r="O13" s="55">
+      <c r="O13" s="27">
         <v>169</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
-      <c r="A14" s="64">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" s="31">
         <v>6</v>
       </c>
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="45">
+      <c r="C14" s="7">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="D14" s="45">
+      <c r="D14" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E14" s="55">
+      <c r="E14" s="27">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="F14" s="54">
+      <c r="F14" s="26">
         <v>4</v>
       </c>
-      <c r="G14" s="45">
-        <v>0</v>
-      </c>
-      <c r="H14" s="45">
+      <c r="G14" s="7">
+        <v>0</v>
+      </c>
+      <c r="H14" s="7">
         <v>9</v>
       </c>
-      <c r="I14" s="45">
-        <v>0</v>
-      </c>
-      <c r="J14" s="45">
+      <c r="I14" s="7">
+        <v>0</v>
+      </c>
+      <c r="J14" s="7">
         <v>30</v>
       </c>
-      <c r="K14" s="45">
-        <v>0</v>
-      </c>
-      <c r="L14" s="45">
-        <v>0</v>
-      </c>
-      <c r="M14" s="45">
-        <v>0</v>
-      </c>
-      <c r="N14" s="45">
+      <c r="K14" s="7">
+        <v>0</v>
+      </c>
+      <c r="L14" s="7">
+        <v>0</v>
+      </c>
+      <c r="M14" s="7">
+        <v>0</v>
+      </c>
+      <c r="N14" s="7">
         <v>2</v>
       </c>
-      <c r="O14" s="55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15">
-      <c r="A15" s="64">
+      <c r="O14" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="31">
         <v>7</v>
       </c>
-      <c r="B15" s="44" t="s">
+      <c r="B15" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="45">
+      <c r="C15" s="7">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D15" s="45">
+      <c r="D15" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E15" s="55">
+      <c r="E15" s="27">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="F15" s="54">
-        <v>0</v>
-      </c>
-      <c r="G15" s="45">
-        <v>0</v>
-      </c>
-      <c r="H15" s="45">
+      <c r="F15" s="26">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7">
+        <v>0</v>
+      </c>
+      <c r="H15" s="7">
         <v>7</v>
       </c>
-      <c r="I15" s="45">
-        <v>0</v>
-      </c>
-      <c r="J15" s="45">
-        <v>0</v>
-      </c>
-      <c r="K15" s="45">
-        <v>0</v>
-      </c>
-      <c r="L15" s="45">
+      <c r="I15" s="7">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7">
+        <v>0</v>
+      </c>
+      <c r="K15" s="7">
+        <v>0</v>
+      </c>
+      <c r="L15" s="7">
         <v>5</v>
       </c>
-      <c r="M15" s="45">
-        <v>0</v>
-      </c>
-      <c r="N15" s="45">
+      <c r="M15" s="7">
+        <v>0</v>
+      </c>
+      <c r="N15" s="7">
         <v>2</v>
       </c>
-      <c r="O15" s="55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15">
-      <c r="A16" s="64">
+      <c r="O15" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="31">
         <v>8</v>
       </c>
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="45">
+      <c r="C16" s="7">
         <f t="shared" si="0"/>
         <v>1588</v>
       </c>
-      <c r="D16" s="45">
+      <c r="D16" s="7">
         <f t="shared" si="1"/>
         <v>1113</v>
       </c>
-      <c r="E16" s="55">
+      <c r="E16" s="27">
         <f t="shared" si="2"/>
         <v>2701</v>
       </c>
-      <c r="F16" s="54">
+      <c r="F16" s="26">
         <v>494</v>
       </c>
-      <c r="G16" s="45">
+      <c r="G16" s="7">
         <v>297</v>
       </c>
-      <c r="H16" s="45">
+      <c r="H16" s="7">
         <v>463</v>
       </c>
-      <c r="I16" s="45">
+      <c r="I16" s="7">
         <v>199</v>
       </c>
-      <c r="J16" s="45">
+      <c r="J16" s="7">
         <v>13</v>
       </c>
-      <c r="K16" s="45">
+      <c r="K16" s="7">
         <v>5</v>
       </c>
-      <c r="L16" s="45">
+      <c r="L16" s="7">
         <v>144</v>
       </c>
-      <c r="M16" s="45">
+      <c r="M16" s="7">
         <v>127</v>
       </c>
-      <c r="N16" s="45">
+      <c r="N16" s="7">
         <v>474</v>
       </c>
-      <c r="O16" s="55">
+      <c r="O16" s="27">
         <v>485</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
-      <c r="A17" s="64">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17" s="31">
         <v>9</v>
       </c>
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="45">
+      <c r="C17" s="7">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D17" s="45">
+      <c r="D17" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E17" s="55">
+      <c r="E17" s="27">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="F17" s="54">
-        <v>0</v>
-      </c>
-      <c r="G17" s="45">
-        <v>0</v>
-      </c>
-      <c r="H17" s="45">
+      <c r="F17" s="26">
+        <v>0</v>
+      </c>
+      <c r="G17" s="7">
+        <v>0</v>
+      </c>
+      <c r="H17" s="7">
         <v>2</v>
       </c>
-      <c r="I17" s="45">
-        <v>0</v>
-      </c>
-      <c r="J17" s="45">
-        <v>0</v>
-      </c>
-      <c r="K17" s="45">
-        <v>0</v>
-      </c>
-      <c r="L17" s="45">
-        <v>0</v>
-      </c>
-      <c r="M17" s="45">
-        <v>0</v>
-      </c>
-      <c r="N17" s="45">
+      <c r="I17" s="7">
+        <v>0</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0</v>
+      </c>
+      <c r="K17" s="7">
+        <v>0</v>
+      </c>
+      <c r="L17" s="7">
+        <v>0</v>
+      </c>
+      <c r="M17" s="7">
+        <v>0</v>
+      </c>
+      <c r="N17" s="7">
         <v>5</v>
       </c>
-      <c r="O17" s="55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15">
-      <c r="A18" s="64">
+      <c r="O17" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18" s="31">
         <v>10</v>
       </c>
-      <c r="B18" s="44" t="s">
+      <c r="B18" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="45">
+      <c r="C18" s="7">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D18" s="45">
+      <c r="D18" s="7">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="E18" s="55">
+      <c r="E18" s="27">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="F18" s="54">
-        <v>0</v>
-      </c>
-      <c r="G18" s="45">
-        <v>0</v>
-      </c>
-      <c r="H18" s="45">
+      <c r="F18" s="26">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7">
+        <v>0</v>
+      </c>
+      <c r="H18" s="7">
         <v>9</v>
       </c>
-      <c r="I18" s="45">
+      <c r="I18" s="7">
         <v>4</v>
       </c>
-      <c r="J18" s="45">
-        <v>0</v>
-      </c>
-      <c r="K18" s="45">
-        <v>0</v>
-      </c>
-      <c r="L18" s="45">
-        <v>0</v>
-      </c>
-      <c r="M18" s="45">
-        <v>0</v>
-      </c>
-      <c r="N18" s="45">
-        <v>0</v>
-      </c>
-      <c r="O18" s="55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15">
-      <c r="A19" s="64">
+      <c r="J18" s="7">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7">
+        <v>0</v>
+      </c>
+      <c r="L18" s="7">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7">
+        <v>0</v>
+      </c>
+      <c r="N18" s="7">
+        <v>0</v>
+      </c>
+      <c r="O18" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" s="31">
         <v>11</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="45">
+      <c r="C19" s="7">
         <f t="shared" si="0"/>
         <v>7556</v>
       </c>
-      <c r="D19" s="45">
+      <c r="D19" s="7">
         <f t="shared" si="1"/>
         <v>13665</v>
       </c>
-      <c r="E19" s="55">
+      <c r="E19" s="27">
         <f t="shared" si="2"/>
         <v>21221</v>
       </c>
-      <c r="F19" s="54">
+      <c r="F19" s="26">
         <v>2121</v>
       </c>
-      <c r="G19" s="45">
+      <c r="G19" s="7">
         <v>2247</v>
       </c>
-      <c r="H19" s="45">
+      <c r="H19" s="7">
         <v>2085</v>
       </c>
-      <c r="I19" s="45">
+      <c r="I19" s="7">
         <v>5822</v>
       </c>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45">
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7">
         <v>1135</v>
       </c>
-      <c r="M19" s="45">
+      <c r="M19" s="7">
         <v>2553</v>
       </c>
-      <c r="N19" s="45">
+      <c r="N19" s="7">
         <v>2215</v>
       </c>
-      <c r="O19" s="55">
+      <c r="O19" s="27">
         <v>3043</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="15.75" thickBot="1">
-      <c r="A20" s="65"/>
-      <c r="B20" s="66"/>
-      <c r="C20" s="57">
-        <f>SUM(C9:C19)</f>
+    <row r="20" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="32"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="29">
+        <f t="shared" ref="C20:O20" si="3">SUM(C9:C19)</f>
         <v>24061</v>
       </c>
-      <c r="D20" s="57">
-        <f>SUM(D9:D19)</f>
+      <c r="D20" s="29">
+        <f t="shared" si="3"/>
         <v>19698</v>
       </c>
-      <c r="E20" s="58">
-        <f>SUM(E9:E19)</f>
+      <c r="E20" s="30">
+        <f t="shared" si="3"/>
         <v>43759</v>
       </c>
-      <c r="F20" s="56">
-        <f>SUM(F9:F19)</f>
+      <c r="F20" s="28">
+        <f t="shared" si="3"/>
         <v>6851</v>
       </c>
-      <c r="G20" s="57">
-        <f>SUM(G9:G19)</f>
+      <c r="G20" s="29">
+        <f t="shared" si="3"/>
         <v>3451</v>
       </c>
-      <c r="H20" s="57">
-        <f>SUM(H9:H19)</f>
+      <c r="H20" s="29">
+        <f t="shared" si="3"/>
         <v>6931</v>
       </c>
-      <c r="I20" s="57">
-        <f>SUM(I9:I19)</f>
+      <c r="I20" s="29">
+        <f t="shared" si="3"/>
         <v>6948</v>
       </c>
-      <c r="J20" s="57">
-        <f>SUM(J9:J19)</f>
+      <c r="J20" s="29">
+        <f t="shared" si="3"/>
         <v>839</v>
       </c>
-      <c r="K20" s="57">
-        <f>SUM(K9:K19)</f>
+      <c r="K20" s="29">
+        <f t="shared" si="3"/>
         <v>177</v>
       </c>
-      <c r="L20" s="57">
-        <f>SUM(L9:L19)</f>
+      <c r="L20" s="29">
+        <f t="shared" si="3"/>
         <v>5208</v>
       </c>
-      <c r="M20" s="57">
-        <f>SUM(M9:M19)</f>
+      <c r="M20" s="29">
+        <f t="shared" si="3"/>
         <v>4987</v>
       </c>
-      <c r="N20" s="57">
-        <f>SUM(N9:N19)</f>
+      <c r="N20" s="29">
+        <f t="shared" si="3"/>
         <v>4232</v>
       </c>
-      <c r="O20" s="58">
-        <f>SUM(O9:O19)</f>
+      <c r="O20" s="30">
+        <f t="shared" si="3"/>
         <v>4135</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="15.75" thickTop="1"/>
-    <row r="22" spans="1:15">
-      <c r="J22" s="92" t="s">
+    <row r="21" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="J22" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="K22" s="92"/>
-      <c r="L22" s="92"/>
-      <c r="M22" s="92"/>
-      <c r="N22" s="92"/>
-      <c r="O22" s="92"/>
-    </row>
-    <row r="23" spans="1:15">
-      <c r="J23" s="92" t="s">
+      <c r="K22" s="57"/>
+      <c r="L22" s="57"/>
+      <c r="M22" s="57"/>
+      <c r="N22" s="57"/>
+      <c r="O22" s="57"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="J23" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="92"/>
-      <c r="L23" s="92"/>
-      <c r="M23" s="92"/>
-      <c r="N23" s="92"/>
-      <c r="O23" s="92"/>
-    </row>
-    <row r="28" spans="1:15">
-      <c r="J28" s="30" t="s">
+      <c r="K23" s="57"/>
+      <c r="L23" s="57"/>
+      <c r="M23" s="57"/>
+      <c r="N23" s="57"/>
+      <c r="O23" s="57"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="J28" s="59" t="s">
         <v>103</v>
       </c>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
-    </row>
-    <row r="29" spans="1:15">
-      <c r="J29" s="92" t="s">
+      <c r="K28" s="59"/>
+      <c r="L28" s="59"/>
+      <c r="M28" s="59"/>
+      <c r="N28" s="59"/>
+      <c r="O28" s="59"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="J29" s="57" t="s">
         <v>101</v>
       </c>
-      <c r="K29" s="92"/>
-      <c r="L29" s="92"/>
-      <c r="M29" s="92"/>
-      <c r="N29" s="92"/>
-      <c r="O29" s="92"/>
+      <c r="K29" s="57"/>
+      <c r="L29" s="57"/>
+      <c r="M29" s="57"/>
+      <c r="N29" s="57"/>
+      <c r="O29" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:O3"/>
     <mergeCell ref="J22:O22"/>
     <mergeCell ref="J23:O23"/>
@@ -3990,185 +3960,186 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:H17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="40.5703125" customWidth="1"/>
-    <col min="3" max="8" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="2" max="2" width="40.5546875" customWidth="1"/>
+    <col min="3" max="8" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" ht="17.25">
-      <c r="A2" s="98" t="s">
+    <row r="2" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A2" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.75">
-      <c r="A4" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="94" t="s">
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="103" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="102" t="s">
         <v>70</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="81" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="95" t="s">
+      <c r="D4" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-    </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1">
-      <c r="A5" s="93"/>
-      <c r="B5" s="94"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="96" t="s">
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="103"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="83"/>
+      <c r="D5" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="96" t="s">
+      <c r="F5" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="96" t="s">
+      <c r="G5" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="96" t="s">
+      <c r="H5" s="44" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1">
-      <c r="A6" s="9">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
         <v>1</v>
       </c>
-      <c r="B6" s="97" t="s">
+      <c r="B6" s="45" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1">
-      <c r="A7" s="9">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7">
         <v>2</v>
       </c>
-      <c r="B7" s="97" t="s">
+      <c r="B7" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1">
-      <c r="A8" s="9">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
         <v>3</v>
       </c>
-      <c r="B8" s="97" t="s">
+      <c r="B8" s="45" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
-      <c r="E10" s="11" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E10" s="79" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="E11" s="11" t="s">
+      <c r="F10" s="79"/>
+      <c r="G10" s="79"/>
+      <c r="H10" s="79"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E11" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="E16" s="10" t="s">
+      <c r="F11" s="79"/>
+      <c r="G11" s="79"/>
+      <c r="H11" s="79"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E16" s="80" t="s">
         <v>103</v>
       </c>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-    </row>
-    <row r="17" spans="5:8">
-      <c r="E17" s="11" t="s">
+      <c r="F16" s="80"/>
+      <c r="G16" s="80"/>
+      <c r="H16" s="80"/>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E17" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
+      <c r="F17" s="79"/>
+      <c r="G17" s="79"/>
+      <c r="H17" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="E10:H10"/>
     <mergeCell ref="E11:H11"/>
     <mergeCell ref="E16:H16"/>
     <mergeCell ref="E17:H17"/>
@@ -4176,8 +4147,6 @@
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="D4:H4"/>
     <mergeCell ref="C4:C5"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="E10:H10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -4185,93 +4154,93 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A2:O27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.5546875" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" ht="17.25">
-      <c r="A2" s="67" t="s">
+    <row r="2" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A2" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-    </row>
-    <row r="4" spans="1:15" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="A4" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="8" t="s">
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="68"/>
+    </row>
+    <row r="4" spans="1:15" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="N4" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="O4" s="8" t="s">
+      <c r="O4" s="6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="30" customHeight="1">
+    <row r="5" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -4288,7 +4257,7 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:15" ht="30" customHeight="1">
+    <row r="6" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4305,7 +4274,7 @@
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="1:15" ht="30" customHeight="1">
+    <row r="7" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4322,7 +4291,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" ht="30" customHeight="1">
+    <row r="8" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -4339,7 +4308,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" ht="30" customHeight="1">
+    <row r="9" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -4356,7 +4325,7 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" ht="30" customHeight="1">
+    <row r="10" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -4373,7 +4342,7 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="30" customHeight="1">
+    <row r="11" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -4390,7 +4359,7 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="30" customHeight="1">
+    <row r="12" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -4407,7 +4376,7 @@
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:15" ht="30" customHeight="1">
+    <row r="13" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -4424,7 +4393,7 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:15" ht="30" customHeight="1">
+    <row r="14" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -4441,7 +4410,7 @@
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:15" ht="30" customHeight="1">
+    <row r="15" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -4458,7 +4427,7 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:15" ht="30" customHeight="1">
+    <row r="16" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4475,7 +4444,7 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="1:15" ht="30" customHeight="1">
+    <row r="17" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4492,7 +4461,7 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="1:15" ht="30" customHeight="1">
+    <row r="18" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -4509,7 +4478,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="1:15" ht="30" customHeight="1">
+    <row r="19" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -4526,37 +4495,37 @@
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
-    <row r="21" spans="1:15">
-      <c r="L21" s="11" t="s">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L21" s="79" t="s">
         <v>100</v>
       </c>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-    </row>
-    <row r="22" spans="1:15">
-      <c r="L22" s="11" t="s">
+      <c r="M21" s="79"/>
+      <c r="N21" s="79"/>
+      <c r="O21" s="79"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L22" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-    </row>
-    <row r="26" spans="1:15">
-      <c r="L26" s="10" t="s">
+      <c r="M22" s="79"/>
+      <c r="N22" s="79"/>
+      <c r="O22" s="79"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L26" s="80" t="s">
         <v>97</v>
       </c>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-    </row>
-    <row r="27" spans="1:15">
-      <c r="L27" s="11" t="s">
+      <c r="M26" s="80"/>
+      <c r="N26" s="80"/>
+      <c r="O26" s="80"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L27" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11"/>
-      <c r="O27" s="11"/>
+      <c r="M27" s="79"/>
+      <c r="N27" s="79"/>
+      <c r="O27" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4572,191 +4541,189 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:E19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="37.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="9.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5">
-      <c r="A2" s="30" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="59" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A4" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="15" t="s">
+    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="60" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15" t="s">
+      <c r="D4" s="60"/>
+      <c r="E4" s="60" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="8" t="s">
+    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="60"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="15"/>
-    </row>
-    <row r="6" spans="1:5" ht="35.1" customHeight="1">
-      <c r="A6" s="9">
+      <c r="E5" s="60"/>
+    </row>
+    <row r="6" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
         <v>1</v>
       </c>
-      <c r="B6" s="97" t="s">
+      <c r="B6" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="100" t="s">
+      <c r="C6" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9" t="s">
+      <c r="D6" s="7"/>
+      <c r="E6" s="7" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="35.1" customHeight="1">
-      <c r="A7" s="9">
+    <row r="7" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7">
         <v>2</v>
       </c>
-      <c r="B7" s="97" t="s">
+      <c r="B7" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="100" t="s">
+      <c r="C7" s="7"/>
+      <c r="D7" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="7" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="35.1" customHeight="1">
-      <c r="A8" s="9">
+    <row r="8" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
         <v>3</v>
       </c>
-      <c r="B8" s="97" t="s">
+      <c r="B8" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="C8" s="100" t="s">
+      <c r="C8" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="7"/>
+      <c r="E8" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="35.1" customHeight="1">
-      <c r="A9" s="9">
+    <row r="9" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
         <v>4</v>
       </c>
-      <c r="B9" s="97" t="s">
+      <c r="B9" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="100" t="s">
+      <c r="C9" s="7"/>
+      <c r="D9" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="35.1" customHeight="1">
-      <c r="A10" s="9">
+    <row r="10" spans="1:5" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
-      <c r="B10" s="97" t="s">
+      <c r="B10" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="100" t="s">
+      <c r="C10" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="100"/>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="46"/>
+      <c r="E10" s="7" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1">
-      <c r="A11" s="39"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="102"/>
-      <c r="D11" s="102"/>
-      <c r="E11" s="39"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="B12" s="99"/>
-      <c r="D12" s="92" t="s">
+    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="21"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="21"/>
+      <c r="D12" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="E12" s="92"/>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="B13" s="99"/>
-      <c r="D13" s="92" t="s">
+      <c r="E12" s="57"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="21"/>
+      <c r="D13" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="92"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="B14" s="99"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="B15" s="99"/>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="B16" s="99"/>
-    </row>
-    <row r="17" spans="2:5">
-      <c r="B17" s="99"/>
-    </row>
-    <row r="18" spans="2:5">
-      <c r="B18" s="99"/>
-      <c r="D18" s="101" t="s">
+      <c r="E13" s="57"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="21"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B15" s="21"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B16" s="21"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B17" s="21"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="21"/>
+      <c r="D18" s="58" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="30"/>
-    </row>
-    <row r="19" spans="2:5">
-      <c r="B19" s="99"/>
-      <c r="D19" s="92" t="s">
+      <c r="E18" s="59"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B19" s="21"/>
+      <c r="D19" s="57" t="s">
         <v>98</v>
       </c>
-      <c r="E19" s="92"/>
+      <c r="E19" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="D12:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>